<commit_message>
fix(w3): 매퍼 XML 오분류 — 부분 문자열 → 루트 요소 판별(isMapperXmlDocument)
W4 위험 Top N 실측에서 발견: maven xdoc 문서 4파일(src/site)이 본문 코드 예제의
'<mapper' 부분 문자열로 mapper-xml 프로그램·MyBatis 모델에 오분류(대형 미도달
파일로 위험 상위 오염). 루트 요소 기반 판별을 mybatis/extract.ts 에 신설하고
parseMapperXml 게이트 + program-inventory·rtm 스캐너 교체.
jpetstore 실측: 프로그램 74→70본, 매퍼 11→7 — crud-matrix·si-프로그램목록 재생성.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/jpetstore-6/.understand-anything/doc-output/07_crud-matrix.xlsx
+++ b/examples/jpetstore-6/.understand-anything/doc-output/07_crud-matrix.xlsx
@@ -844,12 +844,12 @@
       <c r="G20"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="J20"/>
@@ -863,7 +863,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>src/site/xdoc/index.xml:381</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:93, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:104, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:59</t>
         </is>
       </c>
     </row>
@@ -893,12 +893,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="J21"/>
@@ -916,7 +916,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:76, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70, src/site/xdoc/index.xml:381, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:37, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/SequenceMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/SequenceMapper.xml:32</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:76, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:93, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:104, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:59, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:37, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/SequenceMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/SequenceMapper.xml:32</t>
         </is>
       </c>
     </row>
@@ -971,12 +971,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="J23"/>
@@ -990,7 +990,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>src/site/xdoc/index.xml:381, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:37, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:76, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:93, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:104, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:59, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:37, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:76, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(demo): jpetstore 재벤더링 — call-edge resolver(51a0649) 반영 재생성
- 07_crud-matrix·rtm.json·rtm.xlsx·si-단위테스트시나리오: 리졸버 정밀화 반영(과잉 CRUD/인용 축소, 예: 로그인 처리 CRU→R)
- si-실적요약보고서(--weeks 2)·si-위험모듈리포트: 앵커 HEAD(dfbb982) 기준 재생성
- change-impact-analysis.md·impact-overlay.json: 동일 시드 5+생성예측(KakaoLogin, 선례 signon) 재현 — sourceCommit 외 diff 0
- 골든 기준선 rtm.citationCount 64→63 갱신(--update-baseline --yes): 과잉 귀속 인용 1건 제거가 원인, 6지표 100% PASS 유지
- 스위트 green: legacy-core 953 · 루트 297

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/jpetstore-6/.understand-anything/doc-output/07_crud-matrix.xlsx
+++ b/examples/jpetstore-6/.understand-anything/doc-output/07_crud-matrix.xlsx
@@ -306,7 +306,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -327,13 +327,13 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="L4"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -343,7 +343,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:52, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:95, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:114, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:127, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:79, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:102, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:122, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:46</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:52, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:79, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:102, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:122, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36</t>
         </is>
       </c>
     </row>
@@ -380,7 +380,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -401,13 +401,13 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="L6"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -417,7 +417,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:52, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:95, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:114, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:127, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:79, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:102, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:122, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:46</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:52, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:95, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:114, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:127, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -500,13 +500,13 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>R</t>
         </is>
       </c>
       <c r="L9"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>R</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:52, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:95, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:114, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:127, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:79, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:102, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:122, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:46</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/AccountMapper.xml:52, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:46</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:46</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:46, src/main/resources/org/mybatis/jpetstore/mapper/CategoryMapper.xml:35, src/main/resources/org/mybatis/jpetstore/mapper/CategoryMapper.xml:26</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/CategoryMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36</t>
         </is>
       </c>
     </row>
@@ -761,11 +761,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="E18"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>R</t>
@@ -785,7 +781,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47</t>
         </is>
       </c>
     </row>
@@ -798,11 +794,7 @@
       <c r="B19"/>
       <c r="C19"/>
       <c r="D19"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+      <c r="E19"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>R</t>
@@ -826,7 +818,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:36, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:46</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ProductMapper.xml:26</t>
         </is>
       </c>
     </row>
@@ -844,12 +836,12 @@
       <c r="G20"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>R</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>R</t>
         </is>
       </c>
       <c r="J20"/>
@@ -863,7 +855,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:93, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:104, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:59</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:59</t>
         </is>
       </c>
     </row>
@@ -878,27 +870,23 @@
       <c r="D21"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F21"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J21"/>
@@ -916,7 +904,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:76, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:93, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:104, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:59, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:37, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/SequenceMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/SequenceMapper.xml:32</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:76, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:37, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:93, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:104, src/main/resources/org/mybatis/jpetstore/mapper/SequenceMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/SequenceMapper.xml:32</t>
         </is>
       </c>
     </row>
@@ -956,7 +944,7 @@
       <c r="D23"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>R</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -966,17 +954,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>R</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>R</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>R</t>
         </is>
       </c>
       <c r="J23"/>
@@ -990,7 +978,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:93, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:104, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:59, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:37, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:76, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70</t>
+          <t>src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:70, src/main/resources/org/mybatis/jpetstore/mapper/ItemMapper.xml:47, src/main/resources/org/mybatis/jpetstore/mapper/LineItemMapper.xml:26, src/main/resources/org/mybatis/jpetstore/mapper/OrderMapper.xml:26</t>
         </is>
       </c>
     </row>

</xml_diff>